<commit_message>
fix: harden September workbook workflows and release regressions
</commit_message>
<xml_diff>
--- a/tests/fixtures/matter-bulk-update.xlsx
+++ b/tests/fixtures/matter-bulk-update.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matter updates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matter Updates" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,97 +439,97 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Matter Status</t>
+          <t>Matter Description</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Matter Description</t>
+          <t>Client Name</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Client Name</t>
+          <t>Client Code</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Client Code</t>
+          <t>Client Contact Number</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Client Contact Number</t>
+          <t>Client Email</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Client Email</t>
+          <t>Opposing Party Name</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Opposing Party Name</t>
+          <t>Opposing Counsel</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Opposing Counsel</t>
+          <t>Forum</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Forum</t>
+          <t>Court</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Court</t>
+          <t>Court Forum Number</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>Court Forum Number</t>
+          <t>Case Number</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>Case Number</t>
+          <t>Filing Number</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>Filing Number</t>
+          <t>Filing Date</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>Filing Date</t>
+          <t>Matter Owner</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>Matter Owner</t>
+          <t>Assigned Team</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Assigned Team</t>
+          <t>Responsible Lawyer</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>Responsible Lawyer</t>
+          <t>Temporary E-Case Number</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>Temporary E-Case Number</t>
+          <t>CNR Number</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>CNR Number</t>
+          <t>Next Hearing Date</t>
         </is>
       </c>
     </row>
@@ -549,7 +549,7 @@
           <t>Civil</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Updated by the canonical bulk-update path.</t>
         </is>

</xml_diff>